<commit_message>
Update manual test plans after the 2026-10-02 build
Order total without delivery is intended while delivery is free, so
BUG-001 and BUG-D01..D03 are marked not a bug, with question Q-09
about showing a delivery fee that is not charged. BUG-004 (empty
address labels) and BUG-006 (e-mail cannot be saved) are fixed in
this build.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/manual/TezChakana_TestPlan.xlsx
+++ b/docs/manual/TezChakana_TestPlan.xlsx
@@ -6499,7 +6499,7 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>Jami = Mahsulotlar uchun + Yetkazib berish; сумма в списке совпадает с Jami.</t>
+          <t>Пока доставка бесплатная (подтверждено владельцем 2026-10-02): Jami = Mahsulotlar uchun, стоимость доставки в итог не входит. Сумма в списке совпадает с Jami. Если доставку сделают платной — Jami = товары + доставка.</t>
         </is>
       </c>
       <c r="G88" s="9" t="inlineStr">
@@ -6509,7 +6509,7 @@
       </c>
       <c r="H88" s="9" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>±</t>
         </is>
       </c>
       <c r="I88" s="9" t="inlineStr">
@@ -6525,7 +6525,7 @@
       <c r="K88" s="9" t="inlineStr"/>
       <c r="L88" s="10" t="inlineStr">
         <is>
-          <t>BUG-001</t>
+          <t>BUG-001 закрыт как «Не баг»; вопрос Q-09 — как показывать бесплатную доставку</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Новый</t>
+          <t>Не баг</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
@@ -14227,7 +14227,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Новый</t>
+          <t>Закрыт</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
@@ -14345,7 +14345,7 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Новый</t>
+          <t>Закрыт</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -15055,7 +15055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15228,21 +15228,40 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Q-08</t>
+          <t>Q-09</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Есть ли отдельный тестовый аккаунт и тестовая карта с балансом, чтобы не тратить личные средства и данные?</t>
+          <t>Доставка сейчас бесплатная (итог без неё — так задумано), но на оформлении/в заказе показана «Доставка 12 000 / Yetkazib berish 15 000». Показывать «0» или «Bepul»?</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>ORD-*, CARD-04, DET-08</t>
+          <t>ORDH-03, CHK-14</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr"/>
       <c r="E9" s="18" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Q-08</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Есть ли отдельный тестовый аккаунт и тестовая карта с балансом, чтобы не тратить личные средства и данные?</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>ORD-*, CARD-04, DET-08</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr"/>
+      <c r="E10" s="18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>